<commit_message>
read SBDE based on header, added invited/extra status; closes #1197
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/SBDE.xlsx
+++ b/owlcms/src/main/resources/templates/registration/SBDE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\registration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD68300-3437-4B1B-829D-7933A5A3B409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5253F05-AB1C-46AB-9C4F-7A0B818BD76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26175" yWindow="780" windowWidth="23850" windowHeight="13980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Athletes" sheetId="1" r:id="rId1"/>
@@ -151,7 +151,7 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>jx:area(lastCell="V10")</t>
+          <t>jx:area(lastCell="W10")</t>
         </r>
         <r>
           <rPr>
@@ -185,7 +185,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:each(items="athletes" var="l" lastCell="V10")</t>
+jx:each(items="athletes" var="l" lastCell="W10")</t>
         </r>
       </text>
     </comment>
@@ -279,7 +279,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="118">
   <si>
     <t>M/F</t>
   </si>
@@ -627,6 +627,12 @@
   </si>
   <si>
     <t>${l.isoBirth}</t>
+  </si>
+  <si>
+    <t>${l.eligibleForIndividualRanking ? "" : "true"}</t>
+  </si>
+  <si>
+    <t>${t.get("Competition.Invited/Extra")}</t>
   </si>
 </sst>
 </file>
@@ -1354,7 +1360,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1527,6 +1533,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -2270,7 +2279,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jean-François Lamy" refreshedDate="45532.984339236114" createdVersion="8" refreshedVersion="8" recordCount="18" xr:uid="{00000000-000A-0000-FFFF-FFFF09000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jean-François Lamy" refreshedDate="45686.671195601855" createdVersion="8" refreshedVersion="8" recordCount="18" xr:uid="{00000000-000A-0000-FFFF-FFFF09000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G598" sheet="Group Data"/>
   </cacheSource>
@@ -3381,7 +3390,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V157"/>
+  <dimension ref="A1:W157"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
@@ -3398,10 +3407,10 @@
     <col min="12" max="12" width="8" style="1" customWidth="1"/>
     <col min="13" max="16" width="26.5703125" customWidth="1"/>
     <col min="17" max="19" width="14" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="22" max="23" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>28</v>
       </c>
@@ -3429,7 +3438,7 @@
       <c r="R1" s="22"/>
       <c r="S1" s="22"/>
     </row>
-    <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>29</v>
       </c>
@@ -3446,7 +3455,7 @@
       <c r="J2" s="13"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>30</v>
       </c>
@@ -3464,7 +3473,7 @@
       <c r="K3" s="11"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>31</v>
       </c>
@@ -3482,46 +3491,46 @@
       <c r="K4" s="11"/>
       <c r="L4" s="4"/>
     </row>
-    <row r="5" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:22" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="68" t="s">
+    <row r="5" spans="1:23" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:23" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="69" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="69"/>
+      <c r="D6" s="69"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
       <c r="N6" s="66"/>
       <c r="O6" s="66"/>
     </row>
-    <row r="7" spans="1:22" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="68" t="s">
+    <row r="7" spans="1:23" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="68"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="68"/>
-      <c r="J7" s="68"/>
-      <c r="K7" s="68"/>
-      <c r="L7" s="68"/>
-      <c r="M7" s="68"/>
+      <c r="B7" s="69"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="69"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
+      <c r="I7" s="69"/>
+      <c r="J7" s="69"/>
+      <c r="K7" s="69"/>
+      <c r="L7" s="69"/>
+      <c r="M7" s="69"/>
       <c r="N7" s="66"/>
       <c r="O7" s="66"/>
     </row>
-    <row r="8" spans="1:22" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" s="6" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="65"/>
       <c r="B8" s="65"/>
       <c r="C8" s="65"/>
@@ -3538,7 +3547,7 @@
       <c r="N8" s="65"/>
       <c r="O8" s="65"/>
     </row>
-    <row r="9" spans="1:22" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>11</v>
       </c>
@@ -3605,8 +3614,11 @@
       <c r="V9" s="12" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" s="40" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W9" s="68" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" s="40" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="28" t="s">
         <v>20</v>
       </c>
@@ -3673,8 +3685,11 @@
       <c r="V10" s="42" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W10" s="42" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="15"/>
       <c r="C11" s="16"/>
@@ -3697,8 +3712,9 @@
       <c r="T11" s="33"/>
       <c r="U11" s="33"/>
       <c r="V11" s="8"/>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W11" s="8"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="15"/>
       <c r="C12" s="16"/>
@@ -3721,8 +3737,9 @@
       <c r="T12" s="33"/>
       <c r="U12" s="33"/>
       <c r="V12" s="8"/>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W12" s="8"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="15"/>
       <c r="C13" s="16"/>
@@ -3745,8 +3762,9 @@
       <c r="T13" s="33"/>
       <c r="U13" s="33"/>
       <c r="V13" s="8"/>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W13" s="8"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="15"/>
       <c r="C14" s="16"/>
@@ -3769,8 +3787,9 @@
       <c r="T14" s="33"/>
       <c r="U14" s="33"/>
       <c r="V14" s="8"/>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W14" s="8"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="16"/>
@@ -3793,8 +3812,9 @@
       <c r="T15" s="33"/>
       <c r="U15" s="33"/>
       <c r="V15" s="8"/>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W15" s="8"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="16"/>
@@ -3817,8 +3837,9 @@
       <c r="T16" s="33"/>
       <c r="U16" s="33"/>
       <c r="V16" s="8"/>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W16" s="8"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="16"/>
@@ -3841,8 +3862,9 @@
       <c r="T17" s="33"/>
       <c r="U17" s="33"/>
       <c r="V17" s="8"/>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W17" s="8"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="16"/>
@@ -3865,8 +3887,9 @@
       <c r="T18" s="33"/>
       <c r="U18" s="33"/>
       <c r="V18" s="8"/>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W18" s="8"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="16"/>
@@ -3889,8 +3912,9 @@
       <c r="T19" s="33"/>
       <c r="U19" s="33"/>
       <c r="V19" s="8"/>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W19" s="8"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="16"/>
@@ -3913,8 +3937,9 @@
       <c r="T20" s="33"/>
       <c r="U20" s="33"/>
       <c r="V20" s="8"/>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W20" s="8"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="16"/>
@@ -3937,8 +3962,9 @@
       <c r="T21" s="33"/>
       <c r="U21" s="33"/>
       <c r="V21" s="8"/>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W21" s="8"/>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="16"/>
@@ -3961,8 +3987,9 @@
       <c r="T22" s="33"/>
       <c r="U22" s="33"/>
       <c r="V22" s="8"/>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W22" s="8"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="16"/>
@@ -3985,8 +4012,9 @@
       <c r="T23" s="33"/>
       <c r="U23" s="33"/>
       <c r="V23" s="8"/>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W23" s="8"/>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="16"/>
@@ -4009,8 +4037,9 @@
       <c r="T24" s="33"/>
       <c r="U24" s="33"/>
       <c r="V24" s="8"/>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W24" s="8"/>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="15"/>
       <c r="B25" s="15"/>
       <c r="C25" s="16"/>
@@ -4033,8 +4062,9 @@
       <c r="T25" s="33"/>
       <c r="U25" s="33"/>
       <c r="V25" s="8"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W25" s="8"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="15"/>
       <c r="B26" s="15"/>
       <c r="C26" s="16"/>
@@ -4057,8 +4087,9 @@
       <c r="T26" s="33"/>
       <c r="U26" s="33"/>
       <c r="V26" s="8"/>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W26" s="8"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="15"/>
       <c r="B27" s="15"/>
       <c r="C27" s="16"/>
@@ -4081,8 +4112,9 @@
       <c r="T27" s="33"/>
       <c r="U27" s="33"/>
       <c r="V27" s="8"/>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W27" s="8"/>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="15"/>
       <c r="C28" s="16"/>
@@ -4105,8 +4137,9 @@
       <c r="T28" s="33"/>
       <c r="U28" s="33"/>
       <c r="V28" s="8"/>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W28" s="8"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="15"/>
       <c r="C29" s="16"/>
@@ -4129,8 +4162,9 @@
       <c r="T29" s="33"/>
       <c r="U29" s="33"/>
       <c r="V29" s="8"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W29" s="8"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="15"/>
       <c r="C30" s="16"/>
@@ -4153,8 +4187,9 @@
       <c r="T30" s="33"/>
       <c r="U30" s="33"/>
       <c r="V30" s="8"/>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W30" s="8"/>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="15"/>
       <c r="B31" s="15"/>
       <c r="C31" s="16"/>
@@ -4177,8 +4212,9 @@
       <c r="T31" s="33"/>
       <c r="U31" s="33"/>
       <c r="V31" s="8"/>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W31" s="8"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="15"/>
       <c r="B32" s="15"/>
       <c r="C32" s="16"/>
@@ -4201,8 +4237,9 @@
       <c r="T32" s="33"/>
       <c r="U32" s="33"/>
       <c r="V32" s="8"/>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W32" s="8"/>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="15"/>
       <c r="B33" s="15"/>
       <c r="C33" s="16"/>
@@ -4225,8 +4262,9 @@
       <c r="T33" s="33"/>
       <c r="U33" s="33"/>
       <c r="V33" s="8"/>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W33" s="8"/>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="15"/>
       <c r="C34" s="16"/>
@@ -4249,8 +4287,9 @@
       <c r="T34" s="33"/>
       <c r="U34" s="33"/>
       <c r="V34" s="8"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W34" s="8"/>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="15"/>
       <c r="B35" s="15"/>
       <c r="C35" s="16"/>
@@ -4273,8 +4312,9 @@
       <c r="T35" s="33"/>
       <c r="U35" s="33"/>
       <c r="V35" s="8"/>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W35" s="8"/>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="15"/>
       <c r="B36" s="15"/>
       <c r="C36" s="16"/>
@@ -4297,8 +4337,9 @@
       <c r="T36" s="33"/>
       <c r="U36" s="33"/>
       <c r="V36" s="8"/>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W36" s="8"/>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="15"/>
       <c r="B37" s="15"/>
       <c r="C37" s="16"/>
@@ -4321,8 +4362,9 @@
       <c r="T37" s="33"/>
       <c r="U37" s="33"/>
       <c r="V37" s="8"/>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W37" s="8"/>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="15"/>
       <c r="B38" s="15"/>
       <c r="C38" s="16"/>
@@ -4345,8 +4387,9 @@
       <c r="T38" s="33"/>
       <c r="U38" s="33"/>
       <c r="V38" s="8"/>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W38" s="8"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="15"/>
       <c r="B39" s="15"/>
       <c r="C39" s="16"/>
@@ -4369,8 +4412,9 @@
       <c r="T39" s="33"/>
       <c r="U39" s="33"/>
       <c r="V39" s="8"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W39" s="8"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
       <c r="C40" s="16"/>
@@ -4393,8 +4437,9 @@
       <c r="T40" s="33"/>
       <c r="U40" s="33"/>
       <c r="V40" s="8"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W40" s="8"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
       <c r="C41" s="16"/>
@@ -4417,8 +4462,9 @@
       <c r="T41" s="33"/>
       <c r="U41" s="33"/>
       <c r="V41" s="8"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W41" s="8"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="15"/>
       <c r="B42" s="15"/>
       <c r="C42" s="16"/>
@@ -4441,8 +4487,9 @@
       <c r="T42" s="33"/>
       <c r="U42" s="33"/>
       <c r="V42" s="8"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W42" s="8"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
       <c r="C43" s="16"/>
@@ -4465,8 +4512,9 @@
       <c r="T43" s="33"/>
       <c r="U43" s="33"/>
       <c r="V43" s="8"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W43" s="8"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
       <c r="C44" s="16"/>
@@ -4489,8 +4537,9 @@
       <c r="T44" s="33"/>
       <c r="U44" s="33"/>
       <c r="V44" s="8"/>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W44" s="8"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
       <c r="C45" s="16"/>
@@ -4513,8 +4562,9 @@
       <c r="T45" s="33"/>
       <c r="U45" s="33"/>
       <c r="V45" s="8"/>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W45" s="8"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="16"/>
@@ -4537,8 +4587,9 @@
       <c r="T46" s="33"/>
       <c r="U46" s="33"/>
       <c r="V46" s="8"/>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W46" s="8"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="16"/>
@@ -4561,8 +4612,9 @@
       <c r="T47" s="33"/>
       <c r="U47" s="33"/>
       <c r="V47" s="8"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W47" s="8"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="16"/>
@@ -4585,8 +4637,9 @@
       <c r="T48" s="33"/>
       <c r="U48" s="33"/>
       <c r="V48" s="8"/>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W48" s="8"/>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="16"/>
@@ -4609,8 +4662,9 @@
       <c r="T49" s="33"/>
       <c r="U49" s="33"/>
       <c r="V49" s="8"/>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W49" s="8"/>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="15"/>
       <c r="B50" s="15"/>
       <c r="C50" s="16"/>
@@ -4633,8 +4687,9 @@
       <c r="T50" s="33"/>
       <c r="U50" s="33"/>
       <c r="V50" s="8"/>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W50" s="8"/>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="15"/>
       <c r="C51" s="16"/>
@@ -4657,8 +4712,9 @@
       <c r="T51" s="33"/>
       <c r="U51" s="33"/>
       <c r="V51" s="8"/>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W51" s="8"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A52" s="15"/>
       <c r="B52" s="15"/>
       <c r="C52" s="16"/>
@@ -4681,8 +4737,9 @@
       <c r="T52" s="33"/>
       <c r="U52" s="33"/>
       <c r="V52" s="8"/>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W52" s="8"/>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" s="15"/>
       <c r="B53" s="15"/>
       <c r="C53" s="16"/>
@@ -4705,8 +4762,9 @@
       <c r="T53" s="33"/>
       <c r="U53" s="33"/>
       <c r="V53" s="8"/>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W53" s="8"/>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="15"/>
       <c r="B54" s="15"/>
       <c r="C54" s="16"/>
@@ -4729,8 +4787,9 @@
       <c r="T54" s="33"/>
       <c r="U54" s="33"/>
       <c r="V54" s="8"/>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W54" s="8"/>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="15"/>
       <c r="B55" s="15"/>
       <c r="C55" s="16"/>
@@ -4753,8 +4812,9 @@
       <c r="T55" s="33"/>
       <c r="U55" s="33"/>
       <c r="V55" s="8"/>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W55" s="8"/>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A56" s="15"/>
       <c r="B56" s="15"/>
       <c r="C56" s="16"/>
@@ -4777,8 +4837,9 @@
       <c r="T56" s="33"/>
       <c r="U56" s="33"/>
       <c r="V56" s="8"/>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W56" s="8"/>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A57" s="15"/>
       <c r="B57" s="15"/>
       <c r="C57" s="16"/>
@@ -4801,8 +4862,9 @@
       <c r="T57" s="33"/>
       <c r="U57" s="33"/>
       <c r="V57" s="8"/>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W57" s="8"/>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="15"/>
       <c r="B58" s="15"/>
       <c r="C58" s="16"/>
@@ -4825,8 +4887,9 @@
       <c r="T58" s="33"/>
       <c r="U58" s="33"/>
       <c r="V58" s="8"/>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W58" s="8"/>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="15"/>
       <c r="B59" s="15"/>
       <c r="C59" s="16"/>
@@ -4849,8 +4912,9 @@
       <c r="T59" s="33"/>
       <c r="U59" s="33"/>
       <c r="V59" s="8"/>
-    </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W59" s="8"/>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A60" s="15"/>
       <c r="B60" s="15"/>
       <c r="C60" s="16"/>
@@ -4873,8 +4937,9 @@
       <c r="T60" s="33"/>
       <c r="U60" s="33"/>
       <c r="V60" s="8"/>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W60" s="8"/>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A61" s="15"/>
       <c r="B61" s="15"/>
       <c r="C61" s="16"/>
@@ -4897,8 +4962,9 @@
       <c r="T61" s="33"/>
       <c r="U61" s="33"/>
       <c r="V61" s="8"/>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W61" s="8"/>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="15"/>
       <c r="B62" s="15"/>
       <c r="C62" s="16"/>
@@ -4921,8 +4987,9 @@
       <c r="T62" s="33"/>
       <c r="U62" s="33"/>
       <c r="V62" s="8"/>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W62" s="8"/>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="15"/>
       <c r="B63" s="15"/>
       <c r="C63" s="16"/>
@@ -4945,8 +5012,9 @@
       <c r="T63" s="33"/>
       <c r="U63" s="33"/>
       <c r="V63" s="8"/>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W63" s="8"/>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="15"/>
       <c r="B64" s="15"/>
       <c r="C64" s="16"/>
@@ -4969,8 +5037,9 @@
       <c r="T64" s="33"/>
       <c r="U64" s="33"/>
       <c r="V64" s="8"/>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W64" s="8"/>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" s="15"/>
       <c r="B65" s="15"/>
       <c r="C65" s="16"/>
@@ -4993,8 +5062,9 @@
       <c r="T65" s="33"/>
       <c r="U65" s="33"/>
       <c r="V65" s="8"/>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W65" s="8"/>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="15"/>
       <c r="B66" s="15"/>
       <c r="C66" s="16"/>
@@ -5017,8 +5087,9 @@
       <c r="T66" s="33"/>
       <c r="U66" s="33"/>
       <c r="V66" s="8"/>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W66" s="8"/>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A67" s="15"/>
       <c r="B67" s="15"/>
       <c r="C67" s="16"/>
@@ -5041,8 +5112,9 @@
       <c r="T67" s="33"/>
       <c r="U67" s="33"/>
       <c r="V67" s="8"/>
-    </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W67" s="8"/>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A68" s="15"/>
       <c r="B68" s="15"/>
       <c r="C68" s="16"/>
@@ -5065,8 +5137,9 @@
       <c r="T68" s="33"/>
       <c r="U68" s="33"/>
       <c r="V68" s="8"/>
-    </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W68" s="8"/>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A69" s="15"/>
       <c r="B69" s="15"/>
       <c r="C69" s="16"/>
@@ -5089,8 +5162,9 @@
       <c r="T69" s="33"/>
       <c r="U69" s="33"/>
       <c r="V69" s="8"/>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W69" s="8"/>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A70" s="15"/>
       <c r="B70" s="15"/>
       <c r="C70" s="16"/>
@@ -5113,8 +5187,9 @@
       <c r="T70" s="33"/>
       <c r="U70" s="33"/>
       <c r="V70" s="8"/>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W70" s="8"/>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A71" s="15"/>
       <c r="B71" s="15"/>
       <c r="C71" s="16"/>
@@ -5137,8 +5212,9 @@
       <c r="T71" s="33"/>
       <c r="U71" s="33"/>
       <c r="V71" s="8"/>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W71" s="8"/>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" s="15"/>
       <c r="B72" s="15"/>
       <c r="C72" s="16"/>
@@ -5161,8 +5237,9 @@
       <c r="T72" s="33"/>
       <c r="U72" s="33"/>
       <c r="V72" s="8"/>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W72" s="8"/>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A73" s="15"/>
       <c r="B73" s="15"/>
       <c r="C73" s="16"/>
@@ -5185,8 +5262,9 @@
       <c r="T73" s="33"/>
       <c r="U73" s="33"/>
       <c r="V73" s="8"/>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W73" s="8"/>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A74" s="15"/>
       <c r="B74" s="15"/>
       <c r="C74" s="16"/>
@@ -5209,8 +5287,9 @@
       <c r="T74" s="33"/>
       <c r="U74" s="33"/>
       <c r="V74" s="8"/>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W74" s="8"/>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A75" s="15"/>
       <c r="B75" s="15"/>
       <c r="C75" s="16"/>
@@ -5233,8 +5312,9 @@
       <c r="T75" s="33"/>
       <c r="U75" s="33"/>
       <c r="V75" s="8"/>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W75" s="8"/>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A76" s="15"/>
       <c r="B76" s="15"/>
       <c r="C76" s="16"/>
@@ -5257,8 +5337,9 @@
       <c r="T76" s="33"/>
       <c r="U76" s="33"/>
       <c r="V76" s="8"/>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W76" s="8"/>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A77" s="15"/>
       <c r="B77" s="15"/>
       <c r="C77" s="16"/>
@@ -5281,8 +5362,9 @@
       <c r="T77" s="33"/>
       <c r="U77" s="33"/>
       <c r="V77" s="8"/>
-    </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W77" s="8"/>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A78" s="15"/>
       <c r="B78" s="15"/>
       <c r="C78" s="16"/>
@@ -5305,8 +5387,9 @@
       <c r="T78" s="33"/>
       <c r="U78" s="33"/>
       <c r="V78" s="8"/>
-    </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W78" s="8"/>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A79" s="15"/>
       <c r="B79" s="15"/>
       <c r="C79" s="16"/>
@@ -5329,8 +5412,9 @@
       <c r="T79" s="33"/>
       <c r="U79" s="33"/>
       <c r="V79" s="8"/>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W79" s="8"/>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A80" s="15"/>
       <c r="B80" s="15"/>
       <c r="C80" s="16"/>
@@ -5353,8 +5437,9 @@
       <c r="T80" s="33"/>
       <c r="U80" s="33"/>
       <c r="V80" s="8"/>
-    </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W80" s="8"/>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A81" s="15"/>
       <c r="B81" s="15"/>
       <c r="C81" s="16"/>
@@ -5377,8 +5462,9 @@
       <c r="T81" s="33"/>
       <c r="U81" s="33"/>
       <c r="V81" s="8"/>
-    </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W81" s="8"/>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A82" s="15"/>
       <c r="B82" s="15"/>
       <c r="C82" s="16"/>
@@ -5401,8 +5487,9 @@
       <c r="T82" s="33"/>
       <c r="U82" s="33"/>
       <c r="V82" s="8"/>
-    </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W82" s="8"/>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A83" s="15"/>
       <c r="B83" s="15"/>
       <c r="C83" s="16"/>
@@ -5425,8 +5512,9 @@
       <c r="T83" s="33"/>
       <c r="U83" s="33"/>
       <c r="V83" s="8"/>
-    </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W83" s="8"/>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A84" s="15"/>
       <c r="B84" s="15"/>
       <c r="C84" s="16"/>
@@ -5449,8 +5537,9 @@
       <c r="T84" s="33"/>
       <c r="U84" s="33"/>
       <c r="V84" s="8"/>
-    </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W84" s="8"/>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A85" s="15"/>
       <c r="B85" s="15"/>
       <c r="C85" s="16"/>
@@ -5473,8 +5562,9 @@
       <c r="T85" s="33"/>
       <c r="U85" s="33"/>
       <c r="V85" s="8"/>
-    </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W85" s="8"/>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A86" s="15"/>
       <c r="B86" s="15"/>
       <c r="C86" s="16"/>
@@ -5497,8 +5587,9 @@
       <c r="T86" s="33"/>
       <c r="U86" s="33"/>
       <c r="V86" s="8"/>
-    </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W86" s="8"/>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A87" s="15"/>
       <c r="B87" s="15"/>
       <c r="C87" s="16"/>
@@ -5521,8 +5612,9 @@
       <c r="T87" s="33"/>
       <c r="U87" s="33"/>
       <c r="V87" s="8"/>
-    </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W87" s="8"/>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A88" s="15"/>
       <c r="B88" s="15"/>
       <c r="C88" s="16"/>
@@ -5545,8 +5637,9 @@
       <c r="T88" s="33"/>
       <c r="U88" s="33"/>
       <c r="V88" s="8"/>
-    </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W88" s="8"/>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A89" s="15"/>
       <c r="B89" s="15"/>
       <c r="C89" s="16"/>
@@ -5569,8 +5662,9 @@
       <c r="T89" s="33"/>
       <c r="U89" s="33"/>
       <c r="V89" s="8"/>
-    </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W89" s="8"/>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A90" s="15"/>
       <c r="B90" s="15"/>
       <c r="C90" s="16"/>
@@ -5593,8 +5687,9 @@
       <c r="T90" s="33"/>
       <c r="U90" s="33"/>
       <c r="V90" s="8"/>
-    </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W90" s="8"/>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A91" s="15"/>
       <c r="B91" s="15"/>
       <c r="C91" s="16"/>
@@ -5617,8 +5712,9 @@
       <c r="T91" s="33"/>
       <c r="U91" s="33"/>
       <c r="V91" s="8"/>
-    </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W91" s="8"/>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A92" s="15"/>
       <c r="B92" s="15"/>
       <c r="C92" s="16"/>
@@ -5641,8 +5737,9 @@
       <c r="T92" s="33"/>
       <c r="U92" s="33"/>
       <c r="V92" s="8"/>
-    </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W92" s="8"/>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A93" s="15"/>
       <c r="B93" s="15"/>
       <c r="C93" s="16"/>
@@ -5665,8 +5762,9 @@
       <c r="T93" s="33"/>
       <c r="U93" s="33"/>
       <c r="V93" s="8"/>
-    </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W93" s="8"/>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A94" s="15"/>
       <c r="B94" s="15"/>
       <c r="C94" s="16"/>
@@ -5689,8 +5787,9 @@
       <c r="T94" s="33"/>
       <c r="U94" s="33"/>
       <c r="V94" s="8"/>
-    </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W94" s="8"/>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A95" s="15"/>
       <c r="B95" s="15"/>
       <c r="C95" s="16"/>
@@ -5713,8 +5812,9 @@
       <c r="T95" s="33"/>
       <c r="U95" s="33"/>
       <c r="V95" s="8"/>
-    </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W95" s="8"/>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A96" s="15"/>
       <c r="B96" s="15"/>
       <c r="C96" s="16"/>
@@ -5737,8 +5837,9 @@
       <c r="T96" s="33"/>
       <c r="U96" s="33"/>
       <c r="V96" s="8"/>
-    </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W96" s="8"/>
+    </row>
+    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A97" s="15"/>
       <c r="B97" s="15"/>
       <c r="C97" s="16"/>
@@ -5761,8 +5862,9 @@
       <c r="T97" s="33"/>
       <c r="U97" s="33"/>
       <c r="V97" s="8"/>
-    </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W97" s="8"/>
+    </row>
+    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A98" s="15"/>
       <c r="B98" s="15"/>
       <c r="C98" s="16"/>
@@ -5785,8 +5887,9 @@
       <c r="T98" s="33"/>
       <c r="U98" s="33"/>
       <c r="V98" s="8"/>
-    </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W98" s="8"/>
+    </row>
+    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A99" s="15"/>
       <c r="B99" s="15"/>
       <c r="C99" s="16"/>
@@ -5809,8 +5912,9 @@
       <c r="T99" s="33"/>
       <c r="U99" s="33"/>
       <c r="V99" s="8"/>
-    </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W99" s="8"/>
+    </row>
+    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A100" s="15"/>
       <c r="B100" s="15"/>
       <c r="C100" s="16"/>
@@ -5833,8 +5937,9 @@
       <c r="T100" s="33"/>
       <c r="U100" s="33"/>
       <c r="V100" s="8"/>
-    </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W100" s="8"/>
+    </row>
+    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A101" s="15"/>
       <c r="B101" s="15"/>
       <c r="C101" s="16"/>
@@ -5857,8 +5962,9 @@
       <c r="T101" s="33"/>
       <c r="U101" s="33"/>
       <c r="V101" s="8"/>
-    </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W101" s="8"/>
+    </row>
+    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A102" s="15"/>
       <c r="B102" s="15"/>
       <c r="C102" s="16"/>
@@ -5881,8 +5987,9 @@
       <c r="T102" s="33"/>
       <c r="U102" s="33"/>
       <c r="V102" s="8"/>
-    </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W102" s="8"/>
+    </row>
+    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A103" s="15"/>
       <c r="B103" s="15"/>
       <c r="C103" s="16"/>
@@ -5905,8 +6012,9 @@
       <c r="T103" s="33"/>
       <c r="U103" s="33"/>
       <c r="V103" s="8"/>
-    </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W103" s="8"/>
+    </row>
+    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A104" s="15"/>
       <c r="B104" s="15"/>
       <c r="C104" s="16"/>
@@ -5929,8 +6037,9 @@
       <c r="T104" s="33"/>
       <c r="U104" s="33"/>
       <c r="V104" s="8"/>
-    </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W104" s="8"/>
+    </row>
+    <row r="105" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A105" s="15"/>
       <c r="B105" s="15"/>
       <c r="C105" s="16"/>
@@ -5953,8 +6062,9 @@
       <c r="T105" s="33"/>
       <c r="U105" s="33"/>
       <c r="V105" s="8"/>
-    </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W105" s="8"/>
+    </row>
+    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A106" s="15"/>
       <c r="B106" s="15"/>
       <c r="C106" s="16"/>
@@ -5977,8 +6087,9 @@
       <c r="T106" s="33"/>
       <c r="U106" s="33"/>
       <c r="V106" s="8"/>
-    </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W106" s="8"/>
+    </row>
+    <row r="107" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A107" s="15"/>
       <c r="B107" s="15"/>
       <c r="C107" s="16"/>
@@ -6001,8 +6112,9 @@
       <c r="T107" s="33"/>
       <c r="U107" s="33"/>
       <c r="V107" s="8"/>
-    </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W107" s="8"/>
+    </row>
+    <row r="108" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A108" s="15"/>
       <c r="B108" s="15"/>
       <c r="C108" s="16"/>
@@ -6025,8 +6137,9 @@
       <c r="T108" s="33"/>
       <c r="U108" s="33"/>
       <c r="V108" s="8"/>
-    </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W108" s="8"/>
+    </row>
+    <row r="109" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A109" s="15"/>
       <c r="B109" s="15"/>
       <c r="C109" s="16"/>
@@ -6049,8 +6162,9 @@
       <c r="T109" s="33"/>
       <c r="U109" s="33"/>
       <c r="V109" s="8"/>
-    </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W109" s="8"/>
+    </row>
+    <row r="110" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A110" s="15"/>
       <c r="B110" s="15"/>
       <c r="C110" s="16"/>
@@ -6073,8 +6187,9 @@
       <c r="T110" s="33"/>
       <c r="U110" s="33"/>
       <c r="V110" s="8"/>
-    </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W110" s="8"/>
+    </row>
+    <row r="111" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A111" s="15"/>
       <c r="B111" s="15"/>
       <c r="C111" s="16"/>
@@ -6097,8 +6212,9 @@
       <c r="T111" s="33"/>
       <c r="U111" s="33"/>
       <c r="V111" s="8"/>
-    </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W111" s="8"/>
+    </row>
+    <row r="112" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A112" s="15"/>
       <c r="B112" s="15"/>
       <c r="C112" s="16"/>
@@ -6121,8 +6237,9 @@
       <c r="T112" s="33"/>
       <c r="U112" s="33"/>
       <c r="V112" s="8"/>
-    </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W112" s="8"/>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A113" s="15"/>
       <c r="B113" s="15"/>
       <c r="C113" s="16"/>
@@ -6145,8 +6262,9 @@
       <c r="T113" s="33"/>
       <c r="U113" s="33"/>
       <c r="V113" s="8"/>
-    </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W113" s="8"/>
+    </row>
+    <row r="114" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A114" s="15"/>
       <c r="B114" s="15"/>
       <c r="C114" s="16"/>
@@ -6169,8 +6287,9 @@
       <c r="T114" s="33"/>
       <c r="U114" s="33"/>
       <c r="V114" s="8"/>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W114" s="8"/>
+    </row>
+    <row r="115" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A115" s="15"/>
       <c r="B115" s="15"/>
       <c r="C115" s="16"/>
@@ -6193,8 +6312,9 @@
       <c r="T115" s="33"/>
       <c r="U115" s="33"/>
       <c r="V115" s="8"/>
-    </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W115" s="8"/>
+    </row>
+    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A116" s="15"/>
       <c r="B116" s="15"/>
       <c r="C116" s="16"/>
@@ -6217,8 +6337,9 @@
       <c r="T116" s="33"/>
       <c r="U116" s="33"/>
       <c r="V116" s="8"/>
-    </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W116" s="8"/>
+    </row>
+    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A117" s="15"/>
       <c r="B117" s="15"/>
       <c r="C117" s="16"/>
@@ -6241,8 +6362,9 @@
       <c r="T117" s="33"/>
       <c r="U117" s="33"/>
       <c r="V117" s="8"/>
-    </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W117" s="8"/>
+    </row>
+    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A118" s="15"/>
       <c r="B118" s="15"/>
       <c r="C118" s="16"/>
@@ -6265,8 +6387,9 @@
       <c r="T118" s="33"/>
       <c r="U118" s="33"/>
       <c r="V118" s="8"/>
-    </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W118" s="8"/>
+    </row>
+    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A119" s="15"/>
       <c r="B119" s="15"/>
       <c r="C119" s="16"/>
@@ -6289,8 +6412,9 @@
       <c r="T119" s="33"/>
       <c r="U119" s="33"/>
       <c r="V119" s="8"/>
-    </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W119" s="8"/>
+    </row>
+    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A120" s="15"/>
       <c r="B120" s="15"/>
       <c r="C120" s="16"/>
@@ -6313,8 +6437,9 @@
       <c r="T120" s="33"/>
       <c r="U120" s="33"/>
       <c r="V120" s="8"/>
-    </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W120" s="8"/>
+    </row>
+    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A121" s="15"/>
       <c r="B121" s="15"/>
       <c r="C121" s="16"/>
@@ -6337,8 +6462,9 @@
       <c r="T121" s="33"/>
       <c r="U121" s="33"/>
       <c r="V121" s="8"/>
-    </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W121" s="8"/>
+    </row>
+    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A122" s="15"/>
       <c r="B122" s="15"/>
       <c r="C122" s="16"/>
@@ -6361,8 +6487,9 @@
       <c r="T122" s="33"/>
       <c r="U122" s="33"/>
       <c r="V122" s="8"/>
-    </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W122" s="8"/>
+    </row>
+    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A123" s="15"/>
       <c r="B123" s="15"/>
       <c r="C123" s="16"/>
@@ -6385,8 +6512,9 @@
       <c r="T123" s="33"/>
       <c r="U123" s="33"/>
       <c r="V123" s="8"/>
-    </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W123" s="8"/>
+    </row>
+    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A124" s="15"/>
       <c r="B124" s="15"/>
       <c r="C124" s="16"/>
@@ -6409,8 +6537,9 @@
       <c r="T124" s="33"/>
       <c r="U124" s="33"/>
       <c r="V124" s="8"/>
-    </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W124" s="8"/>
+    </row>
+    <row r="125" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A125" s="15"/>
       <c r="B125" s="15"/>
       <c r="C125" s="16"/>
@@ -6433,8 +6562,9 @@
       <c r="T125" s="33"/>
       <c r="U125" s="33"/>
       <c r="V125" s="8"/>
-    </row>
-    <row r="126" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W125" s="8"/>
+    </row>
+    <row r="126" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A126" s="15"/>
       <c r="B126" s="15"/>
       <c r="C126" s="16"/>
@@ -6457,8 +6587,9 @@
       <c r="T126" s="33"/>
       <c r="U126" s="33"/>
       <c r="V126" s="8"/>
-    </row>
-    <row r="127" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W126" s="8"/>
+    </row>
+    <row r="127" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A127" s="15"/>
       <c r="B127" s="15"/>
       <c r="C127" s="16"/>
@@ -6481,8 +6612,9 @@
       <c r="T127" s="33"/>
       <c r="U127" s="33"/>
       <c r="V127" s="8"/>
-    </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W127" s="8"/>
+    </row>
+    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A128" s="15"/>
       <c r="B128" s="15"/>
       <c r="C128" s="16"/>
@@ -6505,8 +6637,9 @@
       <c r="T128" s="33"/>
       <c r="U128" s="33"/>
       <c r="V128" s="8"/>
-    </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W128" s="8"/>
+    </row>
+    <row r="129" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A129" s="15"/>
       <c r="B129" s="15"/>
       <c r="C129" s="16"/>
@@ -6529,8 +6662,9 @@
       <c r="T129" s="33"/>
       <c r="U129" s="33"/>
       <c r="V129" s="8"/>
-    </row>
-    <row r="130" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W129" s="8"/>
+    </row>
+    <row r="130" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A130" s="15"/>
       <c r="B130" s="15"/>
       <c r="C130" s="16"/>
@@ -6553,8 +6687,9 @@
       <c r="T130" s="33"/>
       <c r="U130" s="33"/>
       <c r="V130" s="8"/>
-    </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W130" s="8"/>
+    </row>
+    <row r="131" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A131" s="15"/>
       <c r="B131" s="15"/>
       <c r="C131" s="16"/>
@@ -6577,8 +6712,9 @@
       <c r="T131" s="33"/>
       <c r="U131" s="33"/>
       <c r="V131" s="8"/>
-    </row>
-    <row r="132" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W131" s="8"/>
+    </row>
+    <row r="132" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A132" s="15"/>
       <c r="B132" s="15"/>
       <c r="C132" s="16"/>
@@ -6601,8 +6737,9 @@
       <c r="T132" s="33"/>
       <c r="U132" s="33"/>
       <c r="V132" s="8"/>
-    </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W132" s="8"/>
+    </row>
+    <row r="133" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A133" s="15"/>
       <c r="B133" s="15"/>
       <c r="C133" s="16"/>
@@ -6625,8 +6762,9 @@
       <c r="T133" s="33"/>
       <c r="U133" s="33"/>
       <c r="V133" s="8"/>
-    </row>
-    <row r="134" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W133" s="8"/>
+    </row>
+    <row r="134" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A134" s="15"/>
       <c r="B134" s="15"/>
       <c r="C134" s="16"/>
@@ -6649,8 +6787,9 @@
       <c r="T134" s="33"/>
       <c r="U134" s="33"/>
       <c r="V134" s="8"/>
-    </row>
-    <row r="135" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W134" s="8"/>
+    </row>
+    <row r="135" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A135" s="15"/>
       <c r="B135" s="15"/>
       <c r="C135" s="16"/>
@@ -6673,8 +6812,9 @@
       <c r="T135" s="33"/>
       <c r="U135" s="33"/>
       <c r="V135" s="8"/>
-    </row>
-    <row r="136" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W135" s="8"/>
+    </row>
+    <row r="136" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A136" s="15"/>
       <c r="B136" s="15"/>
       <c r="C136" s="16"/>
@@ -6697,8 +6837,9 @@
       <c r="T136" s="33"/>
       <c r="U136" s="33"/>
       <c r="V136" s="8"/>
-    </row>
-    <row r="137" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W136" s="8"/>
+    </row>
+    <row r="137" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A137" s="15"/>
       <c r="B137" s="15"/>
       <c r="C137" s="16"/>
@@ -6721,8 +6862,9 @@
       <c r="T137" s="33"/>
       <c r="U137" s="33"/>
       <c r="V137" s="8"/>
-    </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W137" s="8"/>
+    </row>
+    <row r="138" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A138" s="15"/>
       <c r="B138" s="15"/>
       <c r="C138" s="16"/>
@@ -6745,8 +6887,9 @@
       <c r="T138" s="33"/>
       <c r="U138" s="33"/>
       <c r="V138" s="8"/>
-    </row>
-    <row r="139" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W138" s="8"/>
+    </row>
+    <row r="139" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A139" s="15"/>
       <c r="B139" s="15"/>
       <c r="C139" s="16"/>
@@ -6769,8 +6912,9 @@
       <c r="T139" s="33"/>
       <c r="U139" s="33"/>
       <c r="V139" s="8"/>
-    </row>
-    <row r="140" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W139" s="8"/>
+    </row>
+    <row r="140" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A140" s="15"/>
       <c r="B140" s="15"/>
       <c r="C140" s="16"/>
@@ -6793,8 +6937,9 @@
       <c r="T140" s="33"/>
       <c r="U140" s="33"/>
       <c r="V140" s="8"/>
-    </row>
-    <row r="141" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W140" s="8"/>
+    </row>
+    <row r="141" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A141" s="15"/>
       <c r="B141" s="15"/>
       <c r="C141" s="16"/>
@@ -6817,8 +6962,9 @@
       <c r="T141" s="33"/>
       <c r="U141" s="33"/>
       <c r="V141" s="8"/>
-    </row>
-    <row r="142" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W141" s="8"/>
+    </row>
+    <row r="142" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A142" s="15"/>
       <c r="B142" s="15"/>
       <c r="C142" s="16"/>
@@ -6841,8 +6987,9 @@
       <c r="T142" s="33"/>
       <c r="U142" s="33"/>
       <c r="V142" s="8"/>
-    </row>
-    <row r="143" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W142" s="8"/>
+    </row>
+    <row r="143" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A143" s="15"/>
       <c r="B143" s="15"/>
       <c r="C143" s="16"/>
@@ -6865,8 +7012,9 @@
       <c r="T143" s="33"/>
       <c r="U143" s="33"/>
       <c r="V143" s="8"/>
-    </row>
-    <row r="144" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W143" s="8"/>
+    </row>
+    <row r="144" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A144" s="15"/>
       <c r="B144" s="15"/>
       <c r="C144" s="16"/>
@@ -6889,8 +7037,9 @@
       <c r="T144" s="33"/>
       <c r="U144" s="33"/>
       <c r="V144" s="8"/>
-    </row>
-    <row r="145" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W144" s="8"/>
+    </row>
+    <row r="145" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A145" s="15"/>
       <c r="B145" s="15"/>
       <c r="C145" s="16"/>
@@ -6913,8 +7062,9 @@
       <c r="T145" s="33"/>
       <c r="U145" s="33"/>
       <c r="V145" s="8"/>
-    </row>
-    <row r="146" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W145" s="8"/>
+    </row>
+    <row r="146" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A146" s="15"/>
       <c r="B146" s="15"/>
       <c r="C146" s="16"/>
@@ -6937,8 +7087,9 @@
       <c r="T146" s="33"/>
       <c r="U146" s="33"/>
       <c r="V146" s="8"/>
-    </row>
-    <row r="147" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W146" s="8"/>
+    </row>
+    <row r="147" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A147" s="15"/>
       <c r="B147" s="15"/>
       <c r="C147" s="16"/>
@@ -6961,8 +7112,9 @@
       <c r="T147" s="33"/>
       <c r="U147" s="33"/>
       <c r="V147" s="8"/>
-    </row>
-    <row r="148" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W147" s="8"/>
+    </row>
+    <row r="148" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A148" s="15"/>
       <c r="B148" s="15"/>
       <c r="C148" s="16"/>
@@ -6985,8 +7137,9 @@
       <c r="T148" s="33"/>
       <c r="U148" s="33"/>
       <c r="V148" s="8"/>
-    </row>
-    <row r="149" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W148" s="8"/>
+    </row>
+    <row r="149" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A149" s="15"/>
       <c r="B149" s="15"/>
       <c r="C149" s="16"/>
@@ -7009,8 +7162,9 @@
       <c r="T149" s="33"/>
       <c r="U149" s="33"/>
       <c r="V149" s="8"/>
-    </row>
-    <row r="150" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W149" s="8"/>
+    </row>
+    <row r="150" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A150" s="15"/>
       <c r="B150" s="15"/>
       <c r="C150" s="16"/>
@@ -7033,8 +7187,9 @@
       <c r="T150" s="33"/>
       <c r="U150" s="33"/>
       <c r="V150" s="8"/>
-    </row>
-    <row r="151" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W150" s="8"/>
+    </row>
+    <row r="151" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A151" s="15"/>
       <c r="B151" s="15"/>
       <c r="C151" s="16"/>
@@ -7057,8 +7212,9 @@
       <c r="T151" s="33"/>
       <c r="U151" s="33"/>
       <c r="V151" s="8"/>
-    </row>
-    <row r="152" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W151" s="8"/>
+    </row>
+    <row r="152" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A152" s="15"/>
       <c r="B152" s="15"/>
       <c r="C152" s="16"/>
@@ -7081,8 +7237,9 @@
       <c r="T152" s="33"/>
       <c r="U152" s="33"/>
       <c r="V152" s="8"/>
-    </row>
-    <row r="153" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W152" s="8"/>
+    </row>
+    <row r="153" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A153" s="15"/>
       <c r="B153" s="15"/>
       <c r="C153" s="16"/>
@@ -7105,8 +7262,9 @@
       <c r="T153" s="33"/>
       <c r="U153" s="33"/>
       <c r="V153" s="8"/>
-    </row>
-    <row r="154" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W153" s="8"/>
+    </row>
+    <row r="154" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A154" s="15"/>
       <c r="B154" s="15"/>
       <c r="C154" s="16"/>
@@ -7129,8 +7287,9 @@
       <c r="T154" s="33"/>
       <c r="U154" s="33"/>
       <c r="V154" s="8"/>
-    </row>
-    <row r="155" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W154" s="8"/>
+    </row>
+    <row r="155" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A155" s="15"/>
       <c r="B155" s="15"/>
       <c r="C155" s="16"/>
@@ -7153,8 +7312,9 @@
       <c r="T155" s="33"/>
       <c r="U155" s="33"/>
       <c r="V155" s="8"/>
-    </row>
-    <row r="156" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W155" s="8"/>
+    </row>
+    <row r="156" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A156" s="15"/>
       <c r="B156" s="15"/>
       <c r="C156" s="16"/>
@@ -7177,8 +7337,9 @@
       <c r="T156" s="33"/>
       <c r="U156" s="33"/>
       <c r="V156" s="8"/>
-    </row>
-    <row r="157" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W156" s="8"/>
+    </row>
+    <row r="157" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A157" s="15"/>
       <c r="B157" s="15"/>
       <c r="C157" s="16"/>
@@ -7201,6 +7362,7 @@
       <c r="T157" s="33"/>
       <c r="U157" s="33"/>
       <c r="V157" s="8"/>
+      <c r="W157" s="8"/>
     </row>
   </sheetData>
   <sheetProtection insertRows="0"/>
@@ -7245,7 +7407,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="I10:J10 I11:J157" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="I10:J157" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="records@federation.org" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -7269,13 +7431,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
     </row>
     <row r="2" spans="1:22" s="36" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
@@ -7447,7 +7609,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="70"/>
+      <c r="A3" s="71"/>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
       <c r="D3" s="48"/>

</xml_diff>

<commit_message>
add IMWA team scoring; closes #1215
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/SBDE.xlsx
+++ b/owlcms/src/main/resources/templates/registration/SBDE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\registration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5253F05-AB1C-46AB-9C4F-7A0B818BD76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CF81EC-69F4-4E76-9B7C-9B45EEEFD981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26175" yWindow="780" windowWidth="23850" windowHeight="13980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Athletes" sheetId="1" r:id="rId1"/>
@@ -208,7 +208,7 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>jx:area(lastCell="V3")</t>
+          <t>jx:area(lastCell="W3")</t>
         </r>
       </text>
     </comment>
@@ -222,7 +222,7 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>jx:each(items="groups" var="g" lastCell="V3")</t>
+          <t>jx:each(items="groups" var="g" lastCell="W3")</t>
         </r>
         <r>
           <rPr>
@@ -279,7 +279,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="120">
   <si>
     <t>M/F</t>
   </si>
@@ -633,6 +633,12 @@
   </si>
   <si>
     <t>${t.get("Competition.Invited/Extra")}</t>
+  </si>
+  <si>
+    <t>${t.get("Competition.masters")}</t>
+  </si>
+  <si>
+    <t>${g.masters}</t>
   </si>
 </sst>
 </file>
@@ -1583,7 +1589,7 @@
     <cellStyle name="Title" xfId="34" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="35" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="89">
+  <dxfs count="83">
     <dxf>
       <font>
         <b/>
@@ -1852,54 +1858,6 @@
           <color theme="4" tint="0.499984740745262"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -2279,7 +2237,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jean-François Lamy" refreshedDate="45686.671195601855" createdVersion="8" refreshedVersion="8" recordCount="18" xr:uid="{00000000-000A-0000-FFFF-FFFF09000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jean-François Lamy" refreshedDate="45736.622832986111" createdVersion="8" refreshedVersion="8" recordCount="18" xr:uid="{00000000-000A-0000-FFFF-FFFF09000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G598" sheet="Group Data"/>
   </cacheSource>
@@ -2762,13 +2720,13 @@
     <i/>
   </colItems>
   <formats count="41">
-    <format dxfId="88">
+    <format dxfId="82">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="87">
+    <format dxfId="81">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2777,7 +2735,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2786,7 +2744,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="78">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2795,7 +2753,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="83">
+    <format dxfId="77">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2804,7 +2762,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2813,7 +2771,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2822,7 +2780,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2831,7 +2789,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2840,7 +2798,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2849,7 +2807,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2858,7 +2816,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2867,7 +2825,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2876,7 +2834,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="74">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2885,7 +2843,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2894,7 +2852,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2903,7 +2861,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2912,7 +2870,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2921,7 +2879,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2930,7 +2888,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2939,7 +2897,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2948,7 +2906,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2957,7 +2915,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2966,7 +2924,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2975,7 +2933,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -2984,7 +2942,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -2993,7 +2951,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -3002,7 +2960,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3011,7 +2969,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -3020,7 +2978,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3029,7 +2987,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -3038,7 +2996,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3047,7 +3005,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -3056,7 +3014,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3065,7 +3023,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1" countASubtotal="1">
@@ -3074,19 +3032,19 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="45">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" offset="A1" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="44">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" offset="A1" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="43">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" offset="A1" fieldPosition="0"/>
     </format>
-    <format dxfId="48">
+    <format dxfId="42">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -7371,38 +7329,8 @@
     <mergeCell ref="A7:M7"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="C10:F10">
-    <cfRule type="expression" dxfId="47" priority="10" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11:F31">
-    <cfRule type="expression" dxfId="46" priority="8" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C32:F52">
-    <cfRule type="expression" dxfId="45" priority="6" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C53:F73">
-    <cfRule type="expression" dxfId="44" priority="5" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C74:F157">
-    <cfRule type="expression" dxfId="43" priority="1" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G10">
-    <cfRule type="expression" dxfId="42" priority="9" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G157">
-    <cfRule type="expression" dxfId="41" priority="7" stopIfTrue="1">
+  <conditionalFormatting sqref="C10:G157">
+    <cfRule type="expression" dxfId="41" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7422,7 +7350,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.42578125" customWidth="1"/>
@@ -7430,7 +7358,7 @@
     <col min="6" max="21" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="70" t="s">
         <v>19</v>
       </c>
@@ -7439,7 +7367,7 @@
       <c r="D1" s="70"/>
       <c r="E1" s="70"/>
     </row>
-    <row r="2" spans="1:22" s="36" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" s="36" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
         <v>3</v>
       </c>
@@ -7506,8 +7434,11 @@
       <c r="V2" s="36" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W2" s="36" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>40</v>
       </c>
@@ -7573,6 +7504,9 @@
       </c>
       <c r="V3" s="1" t="s">
         <v>54</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>